<commit_message>
Errors: Fixed Empty entries
</commit_message>
<xml_diff>
--- a/leads_amusement_parks.xlsx
+++ b/leads_amusement_parks.xlsx
@@ -413,7 +413,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E9"/>
+  <dimension ref="A1:E4"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -467,10 +467,22 @@
       </c>
     </row>
     <row r="3">
-      <c r="A3" t="inlineStr"/>
+      <c r="A3" t="inlineStr">
+        <is>
+          <t>Kashmir Amusement Park</t>
+        </is>
+      </c>
       <c r="B3" t="inlineStr"/>
-      <c r="C3" t="inlineStr"/>
-      <c r="D3" t="inlineStr"/>
+      <c r="C3" t="inlineStr">
+        <is>
+          <t>+92 21 34896611</t>
+        </is>
+      </c>
+      <c r="D3" t="inlineStr">
+        <is>
+          <t>https://www.facebook.com  kashmiramusementpark</t>
+        </is>
+      </c>
       <c r="E3" t="inlineStr">
         <is>
           <t>Karachi</t>
@@ -480,116 +492,21 @@
     <row r="4">
       <c r="A4" t="inlineStr">
         <is>
-          <t>Dragon Roller Coaster | Sindbad</t>
+          <t>Jabees Funland</t>
         </is>
       </c>
       <c r="B4" t="inlineStr"/>
       <c r="C4" t="inlineStr">
         <is>
-          <t>+92 21 34990569</t>
+          <t>+92 35215359</t>
         </is>
       </c>
       <c r="D4" t="inlineStr">
         <is>
-          <t>https://sindbadwl.com</t>
+          <t>http://www.facebook.com  funlandkarachi</t>
         </is>
       </c>
       <c r="E4" t="inlineStr">
-        <is>
-          <t>Karachi</t>
-        </is>
-      </c>
-    </row>
-    <row r="5">
-      <c r="A5" t="inlineStr">
-        <is>
-          <t>Sindbad's Wonderland Amusement Park</t>
-        </is>
-      </c>
-      <c r="B5" t="inlineStr"/>
-      <c r="C5" t="inlineStr">
-        <is>
-          <t>+92 21 34990569</t>
-        </is>
-      </c>
-      <c r="D5" t="inlineStr">
-        <is>
-          <t>http://sindbadwl.com</t>
-        </is>
-      </c>
-      <c r="E5" t="inlineStr">
-        <is>
-          <t>Karachi</t>
-        </is>
-      </c>
-    </row>
-    <row r="6">
-      <c r="A6" t="inlineStr">
-        <is>
-          <t>Kashmir Amusement Park</t>
-        </is>
-      </c>
-      <c r="B6" t="inlineStr"/>
-      <c r="C6" t="inlineStr">
-        <is>
-          <t>+92 21 34896611</t>
-        </is>
-      </c>
-      <c r="D6" t="inlineStr">
-        <is>
-          <t>https://www.facebook.com  kashmiramusementpark</t>
-        </is>
-      </c>
-      <c r="E6" t="inlineStr">
-        <is>
-          <t>Karachi</t>
-        </is>
-      </c>
-    </row>
-    <row r="7">
-      <c r="A7" t="inlineStr"/>
-      <c r="B7" t="inlineStr"/>
-      <c r="C7" t="inlineStr"/>
-      <c r="D7" t="inlineStr"/>
-      <c r="E7" t="inlineStr">
-        <is>
-          <t>Karachi</t>
-        </is>
-      </c>
-    </row>
-    <row r="8">
-      <c r="A8" t="inlineStr">
-        <is>
-          <t>Jabees Funland</t>
-        </is>
-      </c>
-      <c r="B8" t="inlineStr"/>
-      <c r="C8" t="inlineStr">
-        <is>
-          <t>+92 35215359</t>
-        </is>
-      </c>
-      <c r="D8" t="inlineStr">
-        <is>
-          <t>http://www.facebook.com  funlandkarachi</t>
-        </is>
-      </c>
-      <c r="E8" t="inlineStr">
-        <is>
-          <t>Karachi</t>
-        </is>
-      </c>
-    </row>
-    <row r="9">
-      <c r="A9" t="inlineStr"/>
-      <c r="B9" t="inlineStr"/>
-      <c r="C9" t="inlineStr">
-        <is>
-          <t>+92 309 2893448</t>
-        </is>
-      </c>
-      <c r="D9" t="inlineStr"/>
-      <c r="E9" t="inlineStr">
         <is>
           <t>Karachi</t>
         </is>

</xml_diff>